<commit_message>
codescan: add v3.0.0 filespec parsing and hardening
</commit_message>
<xml_diff>
--- a/codescan/demo/codescan_results.xlsx
+++ b/codescan/demo/codescan_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="38" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="47" uniqueCount="30">
   <si>
     <t>condition</t>
   </si>
@@ -37,7 +37,34 @@
     <t>metastatic</t>
   </si>
   <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>Diabetes</t>
+  </si>
+  <si>
+    <t>Hypertension</t>
+  </si>
+  <si>
+    <t>Heart failure</t>
+  </si>
+  <si>
+    <t>COPD</t>
+  </si>
+  <si>
+    <t>Cancer (non-met)</t>
+  </si>
+  <si>
+    <t>Metastatic cancer</t>
+  </si>
+  <si>
     <t>matches</t>
+  </si>
+  <si>
+    <t>total_hits</t>
+  </si>
+  <si>
+    <t>positive_units</t>
   </si>
   <si>
     <t>prevalence</t>
@@ -124,7 +151,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -135,157 +162,208 @@
         <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G1" t="s">
         <v>18</v>
+      </c>
+      <c r="H1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1">
         <v>300</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1">
+        <v>300</v>
+      </c>
+      <c r="F2" s="2">
         <v>60</v>
       </c>
-      <c r="D2" s="2">
+      <c r="G2" s="2">
         <v>55.64541227024273</v>
       </c>
-      <c r="E2" s="2">
+      <c r="H2" s="2">
         <v>64.202100920526277</v>
       </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
+      <c r="I2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1">
         <v>194</v>
       </c>
-      <c r="C3" s="2">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1">
+        <v>194</v>
+      </c>
+      <c r="F3" s="2">
         <v>38.799999999999997</v>
       </c>
-      <c r="D3" s="2">
+      <c r="G3" s="2">
         <v>34.62960293500538</v>
       </c>
-      <c r="E3" s="2">
+      <c r="H3" s="2">
         <v>43.141182291333422</v>
       </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
+      <c r="I3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1">
         <v>48</v>
       </c>
-      <c r="C4" s="2">
+      <c r="D4" s="1"/>
+      <c r="E4" s="1">
+        <v>48</v>
+      </c>
+      <c r="F4" s="2">
         <v>9.5999999999999996</v>
       </c>
-      <c r="D4" s="2">
+      <c r="G4" s="2">
         <v>7.3173504665419093</v>
       </c>
-      <c r="E4" s="2">
+      <c r="H4" s="2">
         <v>12.49869624275153</v>
       </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>19</v>
+      <c r="I4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1">
         <v>149</v>
       </c>
-      <c r="C5" s="2">
+      <c r="D5" s="1"/>
+      <c r="E5" s="1">
+        <v>149</v>
+      </c>
+      <c r="F5" s="2">
         <v>29.800000000000001</v>
       </c>
-      <c r="D5" s="2">
+      <c r="G5" s="2">
         <v>25.957321187843259</v>
       </c>
-      <c r="E5" s="2">
+      <c r="H5" s="2">
         <v>33.950702166803481</v>
       </c>
-      <c r="F5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" t="s">
-        <v>19</v>
+      <c r="I5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J5" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1">
         <v>182</v>
       </c>
-      <c r="C6" s="2">
+      <c r="D6" s="1"/>
+      <c r="E6" s="1">
+        <v>182</v>
+      </c>
+      <c r="F6" s="2">
         <v>36.399999999999999</v>
       </c>
-      <c r="D6" s="2">
+      <c r="G6" s="2">
         <v>32.301143591892647</v>
       </c>
-      <c r="E6" s="2">
+      <c r="H6" s="2">
         <v>40.706238468661589</v>
       </c>
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" t="s">
-        <v>20</v>
+      <c r="I6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="1">
         <v>155</v>
       </c>
-      <c r="C7" s="2">
+      <c r="D7" s="1"/>
+      <c r="E7" s="1">
+        <v>155</v>
+      </c>
+      <c r="F7" s="2">
         <v>31</v>
       </c>
-      <c r="D7" s="2">
+      <c r="G7" s="2">
         <v>27.10389112735686</v>
       </c>
-      <c r="E7" s="2">
+      <c r="H7" s="2">
         <v>35.185833810182153</v>
       </c>
-      <c r="F7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" t="s">
-        <v>19</v>
+      <c r="I7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
msm: rework state management with contract/verify/signature modules
</commit_message>
<xml_diff>
--- a/codescan/demo/codescan_results.xlsx
+++ b/codescan/demo/codescan_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="47" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="45" uniqueCount="28">
   <si>
     <t>condition</t>
   </si>
@@ -68,12 +68,6 @@
   </si>
   <si>
     <t>prevalence</t>
-  </si>
-  <si>
-    <t>ci_low</t>
-  </si>
-  <si>
-    <t>ci_high</t>
   </si>
   <si>
     <t>pattern</t>
@@ -151,7 +145,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -177,13 +171,7 @@
         <v>18</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2">
@@ -203,17 +191,11 @@
       <c r="F2" s="2">
         <v>60</v>
       </c>
-      <c r="G2" s="2">
-        <v>55.64541227024273</v>
-      </c>
-      <c r="H2" s="2">
-        <v>64.202100920526277</v>
-      </c>
-      <c r="I2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" t="s">
-        <v>28</v>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -233,17 +215,11 @@
       <c r="F3" s="2">
         <v>38.799999999999997</v>
       </c>
-      <c r="G3" s="2">
-        <v>34.62960293500538</v>
-      </c>
-      <c r="H3" s="2">
-        <v>43.141182291333422</v>
-      </c>
-      <c r="I3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" t="s">
-        <v>28</v>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -263,17 +239,11 @@
       <c r="F4" s="2">
         <v>9.5999999999999996</v>
       </c>
-      <c r="G4" s="2">
-        <v>7.3173504665419093</v>
-      </c>
-      <c r="H4" s="2">
-        <v>12.49869624275153</v>
-      </c>
-      <c r="I4" t="s">
-        <v>23</v>
-      </c>
-      <c r="J4" t="s">
-        <v>28</v>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -293,17 +263,11 @@
       <c r="F5" s="2">
         <v>29.800000000000001</v>
       </c>
-      <c r="G5" s="2">
-        <v>25.957321187843259</v>
-      </c>
-      <c r="H5" s="2">
-        <v>33.950702166803481</v>
-      </c>
-      <c r="I5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" t="s">
-        <v>28</v>
+      <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="6">
@@ -323,17 +287,11 @@
       <c r="F6" s="2">
         <v>36.399999999999999</v>
       </c>
-      <c r="G6" s="2">
-        <v>32.301143591892647</v>
-      </c>
-      <c r="H6" s="2">
-        <v>40.706238468661589</v>
-      </c>
-      <c r="I6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J6" t="s">
-        <v>29</v>
+      <c r="G6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -353,17 +311,11 @@
       <c r="F7" s="2">
         <v>31</v>
       </c>
-      <c r="G7" s="2">
-        <v>27.10389112735686</v>
-      </c>
-      <c r="H7" s="2">
-        <v>35.185833810182153</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
         <v>26</v>
-      </c>
-      <c r="J7" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>